<commit_message>
connectors insert migration [IN PROGRESS 06-09-26 13:03]
</commit_message>
<xml_diff>
--- a/отфильтрованные данные с вопросами.xlsx
+++ b/отфильтрованные данные с вопросами.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\wg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A808DC99-B079-402F-A69A-79572E9B765C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{918271BF-2656-462F-8853-809D280385E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="400" yWindow="380" windowWidth="24660" windowHeight="14260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -951,7 +951,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -965,14 +965,8 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -980,8 +974,8 @@
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1338,11 +1332,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:W42"/>
   <sheetFormatPr defaultRowHeight="25" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="28.81640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="31" style="2" customWidth="1"/>
     <col min="3" max="3" width="17.7265625" style="2" customWidth="1"/>
     <col min="4" max="4" width="19.36328125" style="2" customWidth="1"/>
     <col min="5" max="5" width="0" hidden="1" customWidth="1"/>
@@ -1423,7 +1418,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:23" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:23" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1188270</v>
       </c>
@@ -1461,7 +1456,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:23" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:23" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1298854</v>
       </c>
@@ -1499,7 +1494,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:23" customFormat="1" ht="77.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:23" customFormat="1" ht="77.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1650914</v>
       </c>
@@ -1531,7 +1526,7 @@
         <v>-32767</v>
       </c>
     </row>
-    <row r="5" spans="1:23" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:23" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1736255</v>
       </c>
@@ -1563,7 +1558,7 @@
         <v>-32767</v>
       </c>
     </row>
-    <row r="6" spans="1:23" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:23" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1879395</v>
       </c>
@@ -1717,21 +1712,21 @@
       <c r="M9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="O9" s="9" t="s">
+      <c r="O9" s="7" t="s">
         <v>25</v>
       </c>
       <c r="P9" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="R9" s="9" t="s">
+      <c r="R9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="T9" s="5" t="s">
+      <c r="T9" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="U9" s="6"/>
-      <c r="V9" s="6"/>
-      <c r="W9" s="6"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="5"/>
+      <c r="W9" s="5"/>
     </row>
     <row r="10" spans="1:23" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
@@ -2062,7 +2057,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1160453</v>
       </c>
@@ -2100,7 +2095,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>66397</v>
       </c>
@@ -2132,7 +2127,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>66398</v>
       </c>
@@ -2164,7 +2159,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>74535</v>
       </c>
@@ -2196,7 +2191,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>90226</v>
       </c>
@@ -2228,7 +2223,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>143051</v>
       </c>
@@ -2260,7 +2255,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>39266</v>
       </c>
@@ -2289,7 +2284,7 @@
         <v>-32767</v>
       </c>
     </row>
-    <row r="24" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>88005</v>
       </c>
@@ -2318,7 +2313,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>89853</v>
       </c>
@@ -2347,7 +2342,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>37781</v>
       </c>
@@ -2373,7 +2368,7 @@
         <v>-32767</v>
       </c>
     </row>
-    <row r="27" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>1616195</v>
       </c>
@@ -2414,7 +2409,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>18323</v>
       </c>
@@ -2452,7 +2447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>6053</v>
       </c>
@@ -2487,7 +2482,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>20056</v>
       </c>
@@ -2519,7 +2514,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>20057</v>
       </c>
@@ -2551,7 +2546,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:18" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>164484</v>
       </c>
@@ -2583,7 +2578,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:23" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:23" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>95191</v>
       </c>
@@ -2612,7 +2607,7 @@
         <v>-32767</v>
       </c>
     </row>
-    <row r="34" spans="1:23" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:23" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>69196</v>
       </c>
@@ -2638,195 +2633,210 @@
         <v>-32767</v>
       </c>
     </row>
-    <row r="35" spans="1:23" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A35">
-        <v>20138</v>
-      </c>
-      <c r="B35" t="s">
+    <row r="35" spans="1:23" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A35" s="2">
+        <v>2</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35" s="2" t="s">
         <v>19</v>
       </c>
       <c r="H35" t="s">
         <v>20</v>
       </c>
-      <c r="K35">
+      <c r="K35" s="2">
         <v>2</v>
       </c>
-      <c r="M35" t="s">
+      <c r="M35" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="O35">
-        <v>20</v>
-      </c>
-      <c r="P35" t="s">
+      <c r="O35" s="2">
+        <v>20</v>
+      </c>
+      <c r="P35" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="R35">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="36" spans="1:23" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A36">
+      <c r="Q35"/>
+      <c r="R35" s="2">
+        <v>20</v>
+      </c>
+      <c r="S35"/>
+    </row>
+    <row r="36" spans="1:23" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A36" s="2">
         <v>20149</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="F36" t="s">
+      <c r="F36" s="2" t="s">
         <v>19</v>
       </c>
       <c r="H36" t="s">
         <v>20</v>
       </c>
-      <c r="K36">
+      <c r="K36" s="2">
         <v>7</v>
       </c>
-      <c r="M36" t="s">
+      <c r="M36" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="O36">
+      <c r="O36" s="2">
         <v>18</v>
       </c>
-      <c r="P36" t="s">
+      <c r="P36" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="R36">
+      <c r="Q36"/>
+      <c r="R36" s="2">
         <v>28</v>
       </c>
-    </row>
-    <row r="37" spans="1:23" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A37">
+      <c r="S36"/>
+    </row>
+    <row r="37" spans="1:23" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A37" s="2">
         <v>20170</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F37" s="2" t="s">
         <v>19</v>
       </c>
       <c r="H37" t="s">
         <v>20</v>
       </c>
-      <c r="K37">
-        <v>20</v>
-      </c>
-      <c r="M37" t="s">
+      <c r="K37" s="2">
+        <v>20</v>
+      </c>
+      <c r="M37" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="O37">
+      <c r="O37" s="2">
         <v>18</v>
       </c>
-      <c r="P37" t="s">
+      <c r="P37" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="R37">
+      <c r="Q37"/>
+      <c r="R37" s="2">
         <v>36</v>
       </c>
-    </row>
-    <row r="38" spans="1:23" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A38">
+      <c r="S37"/>
+    </row>
+    <row r="38" spans="1:23" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="2">
         <v>72719</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="F38" t="s">
+      <c r="F38" s="2" t="s">
         <v>19</v>
       </c>
       <c r="H38" t="s">
         <v>20</v>
       </c>
-      <c r="K38">
+      <c r="K38" s="2">
         <v>4</v>
       </c>
-      <c r="L38">
+      <c r="L38" s="2">
         <v>100</v>
       </c>
-      <c r="M38" t="s">
+      <c r="M38" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="P38" t="s">
+      <c r="P38" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="R38">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="39" spans="1:23" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A39">
+      <c r="Q38"/>
+      <c r="R38" s="2">
+        <v>20</v>
+      </c>
+      <c r="S38"/>
+    </row>
+    <row r="39" spans="1:23" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A39" s="2">
         <v>1372735</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="F39" t="s">
+      <c r="F39" s="2" t="s">
         <v>19</v>
       </c>
       <c r="H39" t="s">
         <v>20</v>
       </c>
-      <c r="K39">
+      <c r="K39" s="2">
         <v>2</v>
       </c>
-      <c r="M39" t="s">
+      <c r="M39" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="O39">
-        <v>20</v>
-      </c>
-      <c r="P39" t="s">
+      <c r="O39" s="2">
+        <v>20</v>
+      </c>
+      <c r="P39" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="R39">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="40" spans="1:23" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="T40" s="4" t="s">
+      <c r="Q39"/>
+      <c r="R39" s="2">
+        <v>20</v>
+      </c>
+      <c r="S39"/>
+    </row>
+    <row r="40" spans="1:23" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="H40"/>
+      <c r="Q40"/>
+      <c r="S40"/>
+      <c r="T40" s="6" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="41" spans="1:23" customFormat="1" ht="86.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B41" s="4" t="s">
+    <row r="41" spans="1:23" ht="86.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B41" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="D41" s="4" t="s">
+      <c r="D41" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="G41" s="7" t="s">
+      <c r="G41" s="8" t="s">
         <v>136</v>
       </c>
       <c r="H41" s="4"/>
-      <c r="I41" s="10"/>
-      <c r="L41" s="4" t="s">
+      <c r="I41" s="5"/>
+      <c r="L41" s="6" t="s">
         <v>132</v>
       </c>
+      <c r="Q41"/>
+      <c r="S41"/>
       <c r="T41" s="8" t="s">
         <v>133</v>
       </c>
@@ -2834,11 +2844,14 @@
       <c r="V41" s="8"/>
       <c r="W41" s="8"/>
     </row>
-    <row r="42" spans="1:23" customFormat="1" ht="82" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="4" t="s">
+    <row r="42" spans="1:23" ht="82" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B42" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="G42" s="7"/>
+      <c r="G42" s="8"/>
+      <c r="H42"/>
+      <c r="Q42"/>
+      <c r="S42"/>
       <c r="T42" s="8" t="s">
         <v>135</v>
       </c>
@@ -2846,7 +2859,15 @@
       <c r="V42" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="G1:G42" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="G1:G42" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters blank="1">
+        <filter val="какие типы можно считать соединителями? Сначала я отобрала только два (просто CON и оптический), потом заметила, что есть знакомый 2рмдт без типа вообще, потом увидела адаптеры, которые вроооде тоже почти соединители. Запутанно"/>
+        <filter val="Соединитель / CON"/>
+        <filter val="Соединитель оптический"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="3">
     <mergeCell ref="T41:W41"/>
     <mergeCell ref="T42:V42"/>

</xml_diff>